<commit_message>
2021-12-01 End of day file push
</commit_message>
<xml_diff>
--- a/SQL Scripts/median data.xlsx
+++ b/SQL Scripts/median data.xlsx
@@ -38,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy/mm/dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd;@"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,12 +49,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -69,9 +75,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -366,7 +373,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -549,15 +556,15 @@
       <c r="F11" t="s">
         <v>3</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="2">
         <f>MEDIAN(G1:G10)</f>
         <v>5.49</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="2">
         <f>MEDIAN(H1:H10)</f>
         <v>4.9649999999999999</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="2">
         <f>MEDIAN(I1:I10)</f>
         <v>5.49</v>
       </c>
@@ -609,6 +616,9 @@
       <c r="C14" s="1">
         <v>44132</v>
       </c>
+      <c r="G14">
+        <v>4.12</v>
+      </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15">
@@ -620,6 +630,13 @@
       <c r="C15" s="1">
         <v>44505</v>
       </c>
+      <c r="G15">
+        <v>4.17</v>
+      </c>
+      <c r="H15">
+        <f>((G15-G14)/2)+G14</f>
+        <v>4.1449999999999996</v>
+      </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16">
@@ -631,8 +648,19 @@
       <c r="C16" s="1">
         <v>44151</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
+      <c r="G16" s="2">
+        <v>5.49</v>
+      </c>
+      <c r="H16">
+        <f>((G16-G15)/2)+G15</f>
+        <v>4.83</v>
+      </c>
+      <c r="I16">
+        <f>((G16-G14) / 2) + G14</f>
+        <v>4.8049999999999997</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16">
       <c r="A17">
         <v>16</v>
       </c>
@@ -642,8 +670,23 @@
       <c r="C17" s="1">
         <v>44152</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
+      <c r="G17">
+        <v>5.76</v>
+      </c>
+      <c r="H17">
+        <f>((G17-G16)/2)+G16</f>
+        <v>5.625</v>
+      </c>
+      <c r="I17">
+        <f>((G17-G15) / 2) + G15</f>
+        <v>4.9649999999999999</v>
+      </c>
+      <c r="J17">
+        <f>((G17-G14)/2)+G14</f>
+        <v>4.9399999999999995</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
       <c r="A18">
         <v>17</v>
       </c>
@@ -653,8 +696,27 @@
       <c r="C18" s="1">
         <v>44153</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
+      <c r="G18">
+        <v>9.36</v>
+      </c>
+      <c r="H18">
+        <f>((G18-G17)/2)+G17</f>
+        <v>7.56</v>
+      </c>
+      <c r="I18">
+        <f>((G18-G16) / 2) + G16</f>
+        <v>7.4249999999999998</v>
+      </c>
+      <c r="J18">
+        <f>((G18-G15)/2)+G15</f>
+        <v>6.7649999999999997</v>
+      </c>
+      <c r="K18">
+        <f>((G18-G14)/2)+G14</f>
+        <v>6.74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16">
       <c r="A19">
         <v>18</v>
       </c>
@@ -663,6 +725,263 @@
       </c>
       <c r="C19" s="1">
         <v>44154</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16">
+      <c r="G20">
+        <v>1.27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16">
+      <c r="G21">
+        <v>1.27</v>
+      </c>
+      <c r="H21">
+        <f>((G21-G20)/2)+G20</f>
+        <v>1.27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16">
+      <c r="G22">
+        <v>3.33</v>
+      </c>
+      <c r="H22">
+        <f>((G22-G21)/2)+G21</f>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I22">
+        <f>((G22-G20) / 2) + G20</f>
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16">
+      <c r="G23">
+        <v>3.33</v>
+      </c>
+      <c r="H23">
+        <f>((G23-G22)/2)+G22</f>
+        <v>3.33</v>
+      </c>
+      <c r="I23">
+        <f>((G23-G21) / 2) + G21</f>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="J23">
+        <f>((G23-G20)/2)+G20</f>
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16">
+      <c r="G24" s="2">
+        <v>4.17</v>
+      </c>
+      <c r="H24">
+        <f>((G24-G23)/2)+G23</f>
+        <v>3.75</v>
+      </c>
+      <c r="I24">
+        <f>((G24-G22) / 2) + G22</f>
+        <v>3.75</v>
+      </c>
+      <c r="J24">
+        <f>((G24-G21)/2)+G21</f>
+        <v>2.7199999999999998</v>
+      </c>
+      <c r="K24">
+        <f>((G24-G20)/2)+G20</f>
+        <v>2.7199999999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16">
+      <c r="G25" s="2">
+        <v>5.76</v>
+      </c>
+      <c r="H25">
+        <f>((G25-G24)/2)+G24</f>
+        <v>4.9649999999999999</v>
+      </c>
+      <c r="I25">
+        <f>((G25-G23) / 2) + G23</f>
+        <v>4.5449999999999999</v>
+      </c>
+      <c r="J25">
+        <f>((G25-G22)/2)+G22</f>
+        <v>4.5449999999999999</v>
+      </c>
+      <c r="K25">
+        <f>((G25-G21)/2)+G21</f>
+        <v>3.5150000000000001</v>
+      </c>
+      <c r="L25">
+        <f>((G25-G20)/2)+G20</f>
+        <v>3.5150000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16">
+      <c r="G26">
+        <v>6.88</v>
+      </c>
+      <c r="H26">
+        <f>((G26-G25)/2)+G25</f>
+        <v>6.32</v>
+      </c>
+      <c r="I26">
+        <f>((G26-G24) / 2) + G24</f>
+        <v>5.5250000000000004</v>
+      </c>
+      <c r="J26">
+        <f>((G26-G23)/2)+G23</f>
+        <v>5.1050000000000004</v>
+      </c>
+      <c r="K26">
+        <f>((G26-G22)/2)+G22</f>
+        <v>5.1050000000000004</v>
+      </c>
+      <c r="L26">
+        <f>((G26-G21)/2)+G21</f>
+        <v>4.0749999999999993</v>
+      </c>
+      <c r="M26">
+        <f>((G26-G20)/2)+G20</f>
+        <v>4.0749999999999993</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16">
+      <c r="G27">
+        <v>6.88</v>
+      </c>
+      <c r="H27">
+        <f>((G27-G26)/2)+G26</f>
+        <v>6.88</v>
+      </c>
+      <c r="I27">
+        <f>((G27-G25) / 2) + G25</f>
+        <v>6.32</v>
+      </c>
+      <c r="J27">
+        <f>((G27-G24)/2)+G24</f>
+        <v>5.5250000000000004</v>
+      </c>
+      <c r="K27">
+        <f>((G27-G23)/2)+G23</f>
+        <v>5.1050000000000004</v>
+      </c>
+      <c r="L27">
+        <f>((G27-G22)/2)+G22</f>
+        <v>5.1050000000000004</v>
+      </c>
+      <c r="M27">
+        <f>((G27-G21)/2)+G21</f>
+        <v>4.0749999999999993</v>
+      </c>
+      <c r="N27">
+        <f>((G27-G20)/2)+G20</f>
+        <v>4.0749999999999993</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16">
+      <c r="G28">
+        <v>9.5399999999999991</v>
+      </c>
+      <c r="H28">
+        <f>((G28-G27)/2)+G27</f>
+        <v>8.2099999999999991</v>
+      </c>
+      <c r="I28">
+        <f>((G28-G26) / 2) + G26</f>
+        <v>8.2099999999999991</v>
+      </c>
+      <c r="J28">
+        <f>((G28-G25)/2)+G25</f>
+        <v>7.6499999999999995</v>
+      </c>
+      <c r="K28">
+        <f>((G28-G24)/2)+G24</f>
+        <v>6.8549999999999995</v>
+      </c>
+      <c r="L28">
+        <f>((G28-G23)/2)+G23</f>
+        <v>6.4349999999999996</v>
+      </c>
+      <c r="M28">
+        <f>((G28-G22)/2)+G22</f>
+        <v>6.4349999999999996</v>
+      </c>
+      <c r="N28">
+        <f>((G28-G21)/2)+G21</f>
+        <v>5.4049999999999994</v>
+      </c>
+      <c r="O28">
+        <f>((G28-G20)/2)+G20</f>
+        <v>5.4049999999999994</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16">
+      <c r="G29">
+        <v>9.5399999999999991</v>
+      </c>
+      <c r="H29">
+        <f>((G29-G28)/2)+G28</f>
+        <v>9.5399999999999991</v>
+      </c>
+      <c r="I29">
+        <f>((G29-G27) / 2) + G27</f>
+        <v>8.2099999999999991</v>
+      </c>
+      <c r="J29">
+        <f>((G29-G26)/2)+G26</f>
+        <v>8.2099999999999991</v>
+      </c>
+      <c r="K29">
+        <f>((G29-G25)/2)+G25</f>
+        <v>7.6499999999999995</v>
+      </c>
+      <c r="L29">
+        <f>((G29-G24)/2)+G24</f>
+        <v>6.8549999999999995</v>
+      </c>
+      <c r="M29">
+        <f>((G29-G23)/2)+G23</f>
+        <v>6.4349999999999996</v>
+      </c>
+      <c r="N29">
+        <f>((G29-G22)/2)+G22</f>
+        <v>6.4349999999999996</v>
+      </c>
+      <c r="O29">
+        <f>((G29-G21)/2)+G21</f>
+        <v>5.4049999999999994</v>
+      </c>
+      <c r="P29">
+        <f>((G29-G20)/2)+G20</f>
+        <v>5.4049999999999994</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16">
+      <c r="G31">
+        <v>4.12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16">
+      <c r="G32" s="2">
+        <v>5.49</v>
+      </c>
+      <c r="H32">
+        <f>((G32-G31)/2)+G31</f>
+        <v>4.8049999999999997</v>
+      </c>
+    </row>
+    <row r="33" spans="7:9">
+      <c r="G33">
+        <v>9.36</v>
+      </c>
+      <c r="H33">
+        <f>((G33-G32)/2)+G32</f>
+        <v>7.4249999999999998</v>
+      </c>
+      <c r="I33">
+        <f>((G33-G31) / 2) + G31</f>
+        <v>6.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>